<commit_message>
Daily auto backup 2026-07-31 17:00
</commit_message>
<xml_diff>
--- a/Debug.xlsx
+++ b/Debug.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LOP2COB\Desktop\TOTAL TIME\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{E85FB79A-EAC6-49B0-A1FA-4FB14C723765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD30581F-9F07-4BFC-B8BB-A7A8388A2C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F4C6FF4C-B294-4D5F-A702-8B946AF198DA}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="58">
   <si>
     <t>defect</t>
   </si>
@@ -55,6 +54,165 @@
   </si>
   <si>
     <t>not added because it doesn’t have a time only estimate of 2H</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> | 11 | Official_SW_Plan_Draft_1388451_Read.mpp | {51d59cf1-4fa9-ea11-ae83-e4a471593ba6} | 2.1.9</t>
+  </si>
+  <si>
+    <t>BM-00094172_003 | 12714252 | V363_MY24.75_SW_Development | 1463556 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00094172_003 | 12714253 | V363_MY24.75_SW_Development | 1463556 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00096778_004 | 12069156 | Ford_V710_eAWD_Release Plan | 1475198 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969681 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00081137_009 | 12865684 | P702 Timeline PMINT | 1423340 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00091219_009 | 13078545 | P736_Timeline_Release_PMint | 1501354 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00103221_009 | 12853374 | P702 MY26 Timeline PMINT | 1500412 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00103221_009 | 12853387 | P702 MY26 Timeline PMINT | 1500412 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00091219_009 | 12962084 | P736_Timeline_Release_PMint | 1501354 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00091219_009 | 12962072 | P736_Timeline_Release_PMint | 1501354 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00091219_009 | 12962088 | P736_Timeline_Release_PMint | 1501354 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00091219_009 | 14610854 | P736_Timeline_Release_PMint | 1501354 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969595 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969608 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969620 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969632 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969644 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969657 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00080788_009 | 12969669 | U725_Project_Plan | 1499430 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00101235_010 | 12969755 | MY26_baseline | 1502593 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00101235_010 | 13078291 | MY26_baseline | 1502593 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00101235_010 | 13078292 | MY26_baseline | 1502593 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00047410_005 | 10087841 | Ford_V710_ESP_2023 | 1397187 | 2.1.9</t>
+  </si>
+  <si>
+    <t>BM-00103425_027 | 13252733 | U725_MY26_Plan | 1510332 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00102067_016 | 13226162 | B2OPD_R18.5.2.7SW | 1509409 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14453004 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00103221_009 | 13270071 | P702 MY26 Timeline PMINT | 1500412 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00103221_009 | 13230379 | P702 MY26 Timeline PMINT | 1500412 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00081137_009 | 13273017 | P702 Timeline PMINT | 1423340 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00090913_008 | 13274611 | SW_Release_Plan | 1512206 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00081137_009 | 13288470 | P702 Timeline PMINT | 1423340 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00101235_010 | 13321896 | MY26_baseline | 1502593 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00094172_003 | 13319320 | V363_MY24.75_SW_Development | 1463556 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00096859_008 | 14869024 | P708_MY27_Plan | 1549314 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00103425_021 | 13147155 | U725_MY25_5 | 1507223 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00101235_010 | 13436402 | MY26_baseline | 1502593 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00101235_010 | 13436403 | MY26_baseline | 1502593 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00091219_009 | 14105246 | P736_Timeline_Release_PMint | 1501354 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 13247040 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14362291 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14362292 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14362293 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14453005 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14453007 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 13247015 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 13247028 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00103221_009 | 14405723 | P702 MY26 Timeline PMINT | 1500412 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00105045_009 | 14453008 | P702_MY27_SW_Timeline | 1510023 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00108205_002 | 14869020 | New MS Project plan | 1549307 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00094172_015 | 15152941 | Ford_ICA3_SW_Baseline_2026 | 1559776 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00113174_005 | 15495241 | Ford_MY30_IPB_S750_MPP | 1570008 | 2.1.9.1</t>
+  </si>
+  <si>
+    <t>BM-00113174_005 | 15495254 | Ford_MY30_IPB_S750_MPP | 1570008 | 2.1.9.1</t>
   </si>
 </sst>
 </file>
@@ -472,7 +630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DF0345E-FB9A-4006-A033-5F67D05FE27E}">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E168"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.1796875" bestFit="1" customWidth="1"/>
@@ -790,6 +948,1480 @@
         <v>8</v>
       </c>
     </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>6961325</v>
+      </c>
+      <c r="B59" t="s">
+        <v>57</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>6961323</v>
+      </c>
+      <c r="B60" t="s">
+        <v>56</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>6932046</v>
+      </c>
+      <c r="B61" t="s">
+        <v>5</v>
+      </c>
+      <c r="C61">
+        <v>85.32</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>6932013</v>
+      </c>
+      <c r="B62" t="s">
+        <v>5</v>
+      </c>
+      <c r="C62">
+        <v>71.75</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>6750618</v>
+      </c>
+      <c r="B63" t="s">
+        <v>29</v>
+      </c>
+      <c r="C63">
+        <v>101.75</v>
+      </c>
+      <c r="D63">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>6750604</v>
+      </c>
+      <c r="B64" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64">
+        <v>47.15</v>
+      </c>
+      <c r="D64">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>6701983</v>
+      </c>
+      <c r="B65" t="s">
+        <v>5</v>
+      </c>
+      <c r="C65">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="D65">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>6667389</v>
+      </c>
+      <c r="B66" t="s">
+        <v>55</v>
+      </c>
+      <c r="C66">
+        <v>462.7</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>6659467</v>
+      </c>
+      <c r="B67" t="s">
+        <v>5</v>
+      </c>
+      <c r="C67">
+        <v>583.79999999999995</v>
+      </c>
+      <c r="D67">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>6318896</v>
+      </c>
+      <c r="B68" t="s">
+        <v>54</v>
+      </c>
+      <c r="C68">
+        <v>149.78</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>6269472</v>
+      </c>
+      <c r="B69" t="s">
+        <v>5</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>6269204</v>
+      </c>
+      <c r="B70" t="s">
+        <v>5</v>
+      </c>
+      <c r="C70">
+        <v>129.35</v>
+      </c>
+      <c r="D70">
+        <v>77.3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>6269200</v>
+      </c>
+      <c r="B71" t="s">
+        <v>5</v>
+      </c>
+      <c r="C71">
+        <v>85.95</v>
+      </c>
+      <c r="D71">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>6211015</v>
+      </c>
+      <c r="B72" t="s">
+        <v>5</v>
+      </c>
+      <c r="C72">
+        <v>405.05</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>6210982</v>
+      </c>
+      <c r="B73" t="s">
+        <v>29</v>
+      </c>
+      <c r="C73">
+        <v>929.2</v>
+      </c>
+      <c r="D73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>6195643</v>
+      </c>
+      <c r="B74" t="s">
+        <v>29</v>
+      </c>
+      <c r="C74">
+        <v>443.7</v>
+      </c>
+      <c r="D74">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75">
+        <v>6172585</v>
+      </c>
+      <c r="B75" t="s">
+        <v>30</v>
+      </c>
+      <c r="C75">
+        <v>1917.39</v>
+      </c>
+      <c r="D75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76">
+        <v>6133802</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77">
+        <v>6133800</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78">
+        <v>6133798</v>
+      </c>
+      <c r="C78">
+        <v>0</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79">
+        <v>6133796</v>
+      </c>
+      <c r="C79">
+        <v>0</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80">
+        <v>6133792</v>
+      </c>
+      <c r="C80">
+        <v>0</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81">
+        <v>6133790</v>
+      </c>
+      <c r="C81">
+        <v>0</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82">
+        <v>6133788</v>
+      </c>
+      <c r="C82">
+        <v>0</v>
+      </c>
+      <c r="D82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83">
+        <v>6133722</v>
+      </c>
+      <c r="B83" t="s">
+        <v>53</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84">
+        <v>6079924</v>
+      </c>
+      <c r="B84" t="s">
+        <v>52</v>
+      </c>
+      <c r="C84">
+        <v>845.23</v>
+      </c>
+      <c r="D84">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85">
+        <v>6063624</v>
+      </c>
+      <c r="B85" t="s">
+        <v>29</v>
+      </c>
+      <c r="C85">
+        <v>33.549999999999997</v>
+      </c>
+      <c r="D85">
+        <v>92.15</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A86">
+        <v>6044649</v>
+      </c>
+      <c r="B86" t="s">
+        <v>51</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A87">
+        <v>6044647</v>
+      </c>
+      <c r="B87" t="s">
+        <v>50</v>
+      </c>
+      <c r="C87">
+        <v>1</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A88">
+        <v>6044588</v>
+      </c>
+      <c r="B88" t="s">
+        <v>49</v>
+      </c>
+      <c r="C88">
+        <v>756.15</v>
+      </c>
+      <c r="D88">
+        <v>68.25</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A89">
+        <v>6044570</v>
+      </c>
+      <c r="B89" t="s">
+        <v>48</v>
+      </c>
+      <c r="C89">
+        <v>2104.48</v>
+      </c>
+      <c r="D89">
+        <v>48.5</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A90">
+        <v>6036607</v>
+      </c>
+      <c r="B90" t="s">
+        <v>38</v>
+      </c>
+      <c r="C90">
+        <v>14</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A91">
+        <v>6031205</v>
+      </c>
+      <c r="C91">
+        <v>0</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A92">
+        <v>6028762</v>
+      </c>
+      <c r="B92" t="s">
+        <v>35</v>
+      </c>
+      <c r="C92">
+        <v>621.45000000000005</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A93">
+        <v>6002206</v>
+      </c>
+      <c r="B93" t="s">
+        <v>40</v>
+      </c>
+      <c r="C93">
+        <v>32.25</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A94">
+        <v>5977873</v>
+      </c>
+      <c r="B94" t="s">
+        <v>38</v>
+      </c>
+      <c r="C94">
+        <v>132.19999999999999</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A95">
+        <v>5938012</v>
+      </c>
+      <c r="B95" t="s">
+        <v>47</v>
+      </c>
+      <c r="C95">
+        <v>873.37</v>
+      </c>
+      <c r="D95">
+        <v>100.25</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A96">
+        <v>5938010</v>
+      </c>
+      <c r="B96" t="s">
+        <v>46</v>
+      </c>
+      <c r="C96">
+        <v>1061.96</v>
+      </c>
+      <c r="D96">
+        <v>269.75</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97">
+        <v>5938008</v>
+      </c>
+      <c r="B97" t="s">
+        <v>45</v>
+      </c>
+      <c r="C97">
+        <v>3821.79</v>
+      </c>
+      <c r="D97">
+        <v>800.42</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98">
+        <v>5938002</v>
+      </c>
+      <c r="B98" t="s">
+        <v>44</v>
+      </c>
+      <c r="C98">
+        <v>193.1</v>
+      </c>
+      <c r="D98">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99">
+        <v>5926884</v>
+      </c>
+      <c r="B99" t="s">
+        <v>5</v>
+      </c>
+      <c r="C99">
+        <v>252.59</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100">
+        <v>5926478</v>
+      </c>
+      <c r="B100" t="s">
+        <v>5</v>
+      </c>
+      <c r="C100">
+        <v>17</v>
+      </c>
+      <c r="D100">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101">
+        <v>5925507</v>
+      </c>
+      <c r="B101" t="s">
+        <v>43</v>
+      </c>
+      <c r="C101">
+        <v>664.87</v>
+      </c>
+      <c r="D101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102">
+        <v>5861140</v>
+      </c>
+      <c r="B102" t="s">
+        <v>5</v>
+      </c>
+      <c r="C102">
+        <v>287.02</v>
+      </c>
+      <c r="D102">
+        <v>138.41999999999999</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103">
+        <v>5806348</v>
+      </c>
+      <c r="B103" t="s">
+        <v>8</v>
+      </c>
+      <c r="C103">
+        <v>3761.6</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104">
+        <v>5770927</v>
+      </c>
+      <c r="B104" t="s">
+        <v>40</v>
+      </c>
+      <c r="C104">
+        <v>144.5</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105">
+        <v>5767229</v>
+      </c>
+      <c r="B105" t="s">
+        <v>5</v>
+      </c>
+      <c r="C105">
+        <v>118.2</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A106">
+        <v>5757449</v>
+      </c>
+      <c r="B106" t="s">
+        <v>42</v>
+      </c>
+      <c r="C106">
+        <v>2621.1</v>
+      </c>
+      <c r="D106">
+        <v>604.03</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A107">
+        <v>5757447</v>
+      </c>
+      <c r="B107" t="s">
+        <v>41</v>
+      </c>
+      <c r="C107">
+        <v>1592.03</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A108">
+        <v>5735436</v>
+      </c>
+      <c r="B108" t="s">
+        <v>30</v>
+      </c>
+      <c r="C108">
+        <v>1288.25</v>
+      </c>
+      <c r="D108">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A109">
+        <v>5722826</v>
+      </c>
+      <c r="B109" t="s">
+        <v>40</v>
+      </c>
+      <c r="C109">
+        <v>72</v>
+      </c>
+      <c r="D109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A110">
+        <v>5715690</v>
+      </c>
+      <c r="B110" t="s">
+        <v>5</v>
+      </c>
+      <c r="C110">
+        <v>271.3</v>
+      </c>
+      <c r="D110">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A111">
+        <v>5715685</v>
+      </c>
+      <c r="B111" t="s">
+        <v>5</v>
+      </c>
+      <c r="C111">
+        <v>43.5</v>
+      </c>
+      <c r="D111">
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A112">
+        <v>5691189</v>
+      </c>
+      <c r="B112" t="s">
+        <v>39</v>
+      </c>
+      <c r="C112">
+        <v>1426.5</v>
+      </c>
+      <c r="D112">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A113">
+        <v>5676413</v>
+      </c>
+      <c r="B113" t="s">
+        <v>38</v>
+      </c>
+      <c r="C113">
+        <v>1336.65</v>
+      </c>
+      <c r="D113">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A114">
+        <v>5673425</v>
+      </c>
+      <c r="B114" t="s">
+        <v>5</v>
+      </c>
+      <c r="C114">
+        <v>20.03</v>
+      </c>
+      <c r="D114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A115">
+        <v>5655888</v>
+      </c>
+      <c r="C115">
+        <v>0</v>
+      </c>
+      <c r="D115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A116">
+        <v>5650491</v>
+      </c>
+      <c r="B116" t="s">
+        <v>37</v>
+      </c>
+      <c r="C116">
+        <v>53.7</v>
+      </c>
+      <c r="D116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A117">
+        <v>5650429</v>
+      </c>
+      <c r="B117" t="s">
+        <v>36</v>
+      </c>
+      <c r="C117">
+        <v>51.5</v>
+      </c>
+      <c r="D117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A118">
+        <v>5643981</v>
+      </c>
+      <c r="B118" t="s">
+        <v>35</v>
+      </c>
+      <c r="C118">
+        <v>603.85</v>
+      </c>
+      <c r="D118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A119">
+        <v>5634293</v>
+      </c>
+      <c r="B119" t="s">
+        <v>5</v>
+      </c>
+      <c r="C119">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A120">
+        <v>5633954</v>
+      </c>
+      <c r="B120" t="s">
+        <v>34</v>
+      </c>
+      <c r="C120">
+        <v>45.31</v>
+      </c>
+      <c r="D120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A121">
+        <v>5621126</v>
+      </c>
+      <c r="B121" t="s">
+        <v>33</v>
+      </c>
+      <c r="C121">
+        <v>97.9</v>
+      </c>
+      <c r="D121">
+        <v>27.25</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A122">
+        <v>5606504</v>
+      </c>
+      <c r="B122" t="s">
+        <v>32</v>
+      </c>
+      <c r="C122">
+        <v>867.86</v>
+      </c>
+      <c r="D122">
+        <v>199.27</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123">
+        <v>5589702</v>
+      </c>
+      <c r="B123" t="s">
+        <v>31</v>
+      </c>
+      <c r="C123">
+        <v>3290.18</v>
+      </c>
+      <c r="D123">
+        <v>572.89</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124">
+        <v>5587328</v>
+      </c>
+      <c r="B124" t="s">
+        <v>30</v>
+      </c>
+      <c r="C124">
+        <v>393.6</v>
+      </c>
+      <c r="D124">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125">
+        <v>5571537</v>
+      </c>
+      <c r="C125">
+        <v>274.5</v>
+      </c>
+      <c r="D125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126">
+        <v>5543806</v>
+      </c>
+      <c r="B126" t="s">
+        <v>29</v>
+      </c>
+      <c r="C126">
+        <v>848.75</v>
+      </c>
+      <c r="D126">
+        <v>122.5</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127">
+        <v>5528829</v>
+      </c>
+      <c r="B127" t="s">
+        <v>28</v>
+      </c>
+      <c r="C127">
+        <v>556.95000000000005</v>
+      </c>
+      <c r="D127">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128">
+        <v>5527537</v>
+      </c>
+      <c r="B128" t="s">
+        <v>8</v>
+      </c>
+      <c r="C128">
+        <v>127.7</v>
+      </c>
+      <c r="D128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129">
+        <v>5490261</v>
+      </c>
+      <c r="B129" t="s">
+        <v>27</v>
+      </c>
+      <c r="C129">
+        <v>0</v>
+      </c>
+      <c r="D129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130">
+        <v>5490259</v>
+      </c>
+      <c r="B130" t="s">
+        <v>26</v>
+      </c>
+      <c r="C130">
+        <v>1595.75</v>
+      </c>
+      <c r="D130">
+        <v>1593.05</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131">
+        <v>5470646</v>
+      </c>
+      <c r="B131" t="s">
+        <v>5</v>
+      </c>
+      <c r="C131">
+        <v>915.52</v>
+      </c>
+      <c r="D131">
+        <v>506.35</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A132">
+        <v>5456353</v>
+      </c>
+      <c r="B132" t="s">
+        <v>8</v>
+      </c>
+      <c r="C132">
+        <v>916.87</v>
+      </c>
+      <c r="D132">
+        <v>179.5</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A133">
+        <v>5439257</v>
+      </c>
+      <c r="B133" t="s">
+        <v>5</v>
+      </c>
+      <c r="C133">
+        <v>51.9</v>
+      </c>
+      <c r="D133">
+        <v>112.5</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A134">
+        <v>5417792</v>
+      </c>
+      <c r="C134">
+        <v>0</v>
+      </c>
+      <c r="D134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A135">
+        <v>5407094</v>
+      </c>
+      <c r="B135" t="s">
+        <v>25</v>
+      </c>
+      <c r="C135">
+        <v>2757.45</v>
+      </c>
+      <c r="D135">
+        <v>2451.48</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A136">
+        <v>5407069</v>
+      </c>
+      <c r="B136" t="s">
+        <v>24</v>
+      </c>
+      <c r="C136">
+        <v>0</v>
+      </c>
+      <c r="D136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A137">
+        <v>5407067</v>
+      </c>
+      <c r="B137" t="s">
+        <v>23</v>
+      </c>
+      <c r="C137">
+        <v>0</v>
+      </c>
+      <c r="D137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A138">
+        <v>5407065</v>
+      </c>
+      <c r="B138" t="s">
+        <v>22</v>
+      </c>
+      <c r="C138">
+        <v>0</v>
+      </c>
+      <c r="D138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A139">
+        <v>5407063</v>
+      </c>
+      <c r="B139" t="s">
+        <v>21</v>
+      </c>
+      <c r="C139">
+        <v>0</v>
+      </c>
+      <c r="D139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A140">
+        <v>5407061</v>
+      </c>
+      <c r="B140" t="s">
+        <v>20</v>
+      </c>
+      <c r="C140">
+        <v>0</v>
+      </c>
+      <c r="D140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A141">
+        <v>5407059</v>
+      </c>
+      <c r="B141" t="s">
+        <v>19</v>
+      </c>
+      <c r="C141">
+        <v>0</v>
+      </c>
+      <c r="D141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A142">
+        <v>5407057</v>
+      </c>
+      <c r="B142" t="s">
+        <v>18</v>
+      </c>
+      <c r="C142">
+        <v>0</v>
+      </c>
+      <c r="D142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A143">
+        <v>5407052</v>
+      </c>
+      <c r="C143">
+        <v>0</v>
+      </c>
+      <c r="D143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A144">
+        <v>5407050</v>
+      </c>
+      <c r="C144">
+        <v>0</v>
+      </c>
+      <c r="D144">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A145">
+        <v>5407048</v>
+      </c>
+      <c r="C145">
+        <v>0</v>
+      </c>
+      <c r="D145">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A146">
+        <v>5407046</v>
+      </c>
+      <c r="C146">
+        <v>0</v>
+      </c>
+      <c r="D146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A147">
+        <v>5407044</v>
+      </c>
+      <c r="C147">
+        <v>0</v>
+      </c>
+      <c r="D147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A148">
+        <v>5407042</v>
+      </c>
+      <c r="C148">
+        <v>0</v>
+      </c>
+      <c r="D148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149">
+        <v>5407040</v>
+      </c>
+      <c r="C149">
+        <v>0</v>
+      </c>
+      <c r="D149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150">
+        <v>5407038</v>
+      </c>
+      <c r="C150">
+        <v>0</v>
+      </c>
+      <c r="D150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151">
+        <v>5402012</v>
+      </c>
+      <c r="B151" t="s">
+        <v>17</v>
+      </c>
+      <c r="C151">
+        <v>0</v>
+      </c>
+      <c r="D151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152">
+        <v>5402010</v>
+      </c>
+      <c r="B152" t="s">
+        <v>16</v>
+      </c>
+      <c r="C152">
+        <v>63</v>
+      </c>
+      <c r="D152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A153">
+        <v>5402008</v>
+      </c>
+      <c r="B153" t="s">
+        <v>15</v>
+      </c>
+      <c r="C153">
+        <v>1</v>
+      </c>
+      <c r="D153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A154">
+        <v>5395368</v>
+      </c>
+      <c r="B154" t="s">
+        <v>14</v>
+      </c>
+      <c r="C154">
+        <v>356</v>
+      </c>
+      <c r="D154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A155">
+        <v>5366162</v>
+      </c>
+      <c r="C155">
+        <v>0</v>
+      </c>
+      <c r="D155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A156">
+        <v>5366160</v>
+      </c>
+      <c r="C156">
+        <v>0</v>
+      </c>
+      <c r="D156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A157">
+        <v>5366157</v>
+      </c>
+      <c r="B157" t="s">
+        <v>13</v>
+      </c>
+      <c r="C157">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="D157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A158">
+        <v>5366155</v>
+      </c>
+      <c r="B158" t="s">
+        <v>12</v>
+      </c>
+      <c r="C158">
+        <v>0</v>
+      </c>
+      <c r="D158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A159">
+        <v>5363156</v>
+      </c>
+      <c r="B159" t="s">
+        <v>11</v>
+      </c>
+      <c r="C159">
+        <v>937.75</v>
+      </c>
+      <c r="D159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A160">
+        <v>5355943</v>
+      </c>
+      <c r="B160" t="s">
+        <v>10</v>
+      </c>
+      <c r="C160">
+        <v>121.1</v>
+      </c>
+      <c r="D160">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A161">
+        <v>5320933</v>
+      </c>
+      <c r="C161">
+        <v>198.85</v>
+      </c>
+      <c r="D161">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A162">
+        <v>5312810</v>
+      </c>
+      <c r="B162" t="s">
+        <v>9</v>
+      </c>
+      <c r="C162">
+        <v>289.14999999999998</v>
+      </c>
+      <c r="D162">
+        <v>115.5</v>
+      </c>
+    </row>
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A163">
+        <v>5305988</v>
+      </c>
+      <c r="B163" t="s">
+        <v>8</v>
+      </c>
+      <c r="C163">
+        <v>1456.63</v>
+      </c>
+      <c r="D163">
+        <v>613.33000000000004</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A164">
+        <v>5305839</v>
+      </c>
+      <c r="B164" t="s">
+        <v>8</v>
+      </c>
+      <c r="C164">
+        <v>1237.47</v>
+      </c>
+      <c r="D164">
+        <v>75.5</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A165">
+        <v>5267139</v>
+      </c>
+      <c r="B165" t="s">
+        <v>8</v>
+      </c>
+      <c r="C165">
+        <v>3364.97</v>
+      </c>
+      <c r="D165">
+        <v>781.53</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A166">
+        <v>5266715</v>
+      </c>
+      <c r="B166" t="s">
+        <v>7</v>
+      </c>
+      <c r="C166">
+        <v>870.22</v>
+      </c>
+      <c r="D166">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A167">
+        <v>5266712</v>
+      </c>
+      <c r="B167" t="s">
+        <v>6</v>
+      </c>
+      <c r="C167">
+        <v>2806.37</v>
+      </c>
+      <c r="D167">
+        <v>331.5</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A168">
+        <v>5266012</v>
+      </c>
+      <c r="B168" t="s">
+        <v>5</v>
+      </c>
+      <c r="C168">
+        <v>133.5</v>
+      </c>
+      <c r="D168">
+        <v>171</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>